<commit_message>
création bilan général suivi Collection HAL
</commit_message>
<xml_diff>
--- a/Data/Suivi_Démarche_questionnaires.xlsx
+++ b/Data/Suivi_Démarche_questionnaires.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dutroncj\Documents\Outils\FairCarboN_datas\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D67F404-4C89-4E2C-A474-97919347E481}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF83635A-69DE-42C2-821F-A781553DB8A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="175">
   <si>
     <t>1.2 Incertitudes</t>
   </si>
@@ -240,16 +240,10 @@
     <t>Benoit.Gaudou@ut-capitole.fr</t>
   </si>
   <si>
-    <t>patrice.buche@inrae.fr</t>
-  </si>
-  <si>
     <t>jonathan.vayssieres@cirad.Fr</t>
   </si>
   <si>
     <t>olivier.therond@inrae.fr</t>
-  </si>
-  <si>
-    <t>petros.chatzimpiros@u-paris.fr</t>
   </si>
   <si>
     <t>antonello.lobianco@inrae.fr</t>
@@ -375,11 +369,6 @@
   <si>
     <t>baptistelesquoy@protonmail.com
 alexis.drogoul@ird.fr</t>
-  </si>
-  <si>
-    <t>wafa.malik@cirad.fr
-gabin.guillemaud@inrae.fr
-eleonore.loiseau@inrae.fr</t>
   </si>
   <si>
     <t>jeremy.pantet@inrae.fr
@@ -518,9 +507,6 @@
     <t>Intitulés données</t>
   </si>
   <si>
-    <t>AD RESULTS</t>
-  </si>
-  <si>
     <t>scenario enr</t>
   </si>
   <si>
@@ -582,6 +568,55 @@
   </si>
   <si>
     <t>environ 50 noms</t>
+  </si>
+  <si>
+    <t>Relances_post_début</t>
+  </si>
+  <si>
+    <t>AD RESULTS
+FAIRCARBON SLAM-B PROPOSAL
+SCENARIO LABS INFO</t>
+  </si>
+  <si>
+    <t>Wasim Ahmed (côté logiciel)</t>
+  </si>
+  <si>
+    <t>Tiziano</t>
+  </si>
+  <si>
+    <t>patrice.buche@inrae.fr
+florian.goutieras@inrae.fr</t>
+  </si>
+  <si>
+    <t>Florian Goutieras</t>
+  </si>
+  <si>
+    <t>envoi questionnaires à la seconde relance</t>
+  </si>
+  <si>
+    <t>petros.chatzimpiros@u-paris.fr
+souhil.harchaoui@inrae.fr</t>
+  </si>
+  <si>
+    <t>Simon Charrière principalement</t>
+  </si>
+  <si>
+    <t>Souhil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Antonello </t>
+  </si>
+  <si>
+    <t>wafa.malik@cirad.fr
+gabin.guillemaud@inrae.fr
+eleonore.loiseau@inrae.fr
+julie.auberger@inrae.fr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eleonore, julie </t>
+  </si>
+  <si>
+    <t>kevin</t>
   </si>
 </sst>
 </file>
@@ -662,7 +697,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -711,6 +746,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -740,7 +781,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -827,6 +868,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1130,12 +1174,13 @@
     <col min="17" max="17" width="36.1796875" style="18" customWidth="1"/>
     <col min="18" max="18" width="17.90625" style="18" customWidth="1"/>
     <col min="19" max="19" width="68.08984375" style="18" customWidth="1"/>
-    <col min="20" max="21" width="9.1796875" style="4"/>
+    <col min="20" max="20" width="27.26953125" style="4" customWidth="1"/>
+    <col min="21" max="21" width="9.1796875" style="4"/>
     <col min="22" max="22" width="12.08984375" style="4" customWidth="1"/>
     <col min="23" max="16384" width="9.1796875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="37" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:20" ht="37" x14ac:dyDescent="0.35">
       <c r="A1" s="28" t="s">
         <v>26</v>
       </c>
@@ -1149,52 +1194,55 @@
         <v>59</v>
       </c>
       <c r="E1" s="28" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F1" s="28" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G1" s="28" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H1" s="28" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I1" s="28" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J1" s="14" t="s">
+        <v>130</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="L1" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="M1" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="N1" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="O1" s="27" t="s">
+        <v>132</v>
+      </c>
+      <c r="P1" s="26" t="s">
+        <v>151</v>
+      </c>
+      <c r="Q1" s="27" t="s">
         <v>133</v>
       </c>
-      <c r="K1" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="L1" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="M1" s="14" t="s">
-        <v>142</v>
-      </c>
-      <c r="N1" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="O1" s="27" t="s">
-        <v>135</v>
-      </c>
-      <c r="P1" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="Q1" s="27" t="s">
-        <v>136</v>
-      </c>
       <c r="R1" s="27" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="S1" s="27" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="2" spans="1:19" ht="21" customHeight="1" x14ac:dyDescent="0.35">
+        <v>153</v>
+      </c>
+      <c r="T1" s="30" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" ht="21" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
         <v>23</v>
       </c>
@@ -1216,8 +1264,9 @@
       <c r="Q2" s="15"/>
       <c r="R2" s="15"/>
       <c r="S2" s="15"/>
-    </row>
-    <row r="3" spans="1:19" ht="29" x14ac:dyDescent="0.35">
+      <c r="T2" s="6"/>
+    </row>
+    <row r="3" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
         <v>1</v>
       </c>
@@ -1231,22 +1280,22 @@
         <v>60</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G3" s="3">
         <v>0</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="J3" s="13" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="K3" s="12">
         <v>1</v>
@@ -1271,8 +1320,11 @@
         <v>0.2</v>
       </c>
       <c r="S3" s="13"/>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="T3" s="7" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -1286,16 +1338,16 @@
         <v>60</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G4" s="8">
         <v>1</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="I4" s="9" t="s">
         <v>65</v>
@@ -1312,8 +1364,9 @@
       <c r="Q4" s="13"/>
       <c r="R4" s="13"/>
       <c r="S4" s="13"/>
-    </row>
-    <row r="5" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="T4" s="7"/>
+    </row>
+    <row r="5" spans="1:20" ht="58" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
         <v>2</v>
       </c>
@@ -1327,22 +1380,22 @@
         <v>61</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G5" s="3">
         <v>0</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>109</v>
+        <v>172</v>
       </c>
       <c r="J5" s="16" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="K5" s="12">
         <v>2</v>
@@ -1351,18 +1404,21 @@
         <v>1.2</v>
       </c>
       <c r="M5" s="13" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="N5" s="13" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="O5" s="16"/>
       <c r="P5" s="12"/>
       <c r="Q5" s="13"/>
       <c r="R5" s="13"/>
       <c r="S5" s="13"/>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="T5" s="7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
         <v>3</v>
       </c>
@@ -1376,19 +1432,19 @@
         <v>61</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G6" s="3">
         <v>1</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>66</v>
+        <v>165</v>
       </c>
       <c r="J6" s="16"/>
       <c r="K6" s="12">
@@ -1402,8 +1458,11 @@
       <c r="Q6" s="13"/>
       <c r="R6" s="13"/>
       <c r="S6" s="13"/>
-    </row>
-    <row r="7" spans="1:19" ht="29" x14ac:dyDescent="0.35">
+      <c r="T6" s="7" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
         <v>4</v>
       </c>
@@ -1417,37 +1476,37 @@
         <v>61</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G7" s="3">
         <v>1</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="K7" s="12">
         <v>1</v>
       </c>
       <c r="L7" s="13">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="M7" s="13">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="N7" s="13" t="s">
-        <v>144</v>
+        <v>162</v>
       </c>
       <c r="O7" s="13" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="P7" s="12">
         <v>1</v>
@@ -1459,10 +1518,13 @@
         <v>0.2</v>
       </c>
       <c r="S7" s="13" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
+        <v>154</v>
+      </c>
+      <c r="T7" s="7" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
         <v>5</v>
       </c>
@@ -1476,19 +1538,19 @@
         <v>61</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G8" s="8">
         <v>1</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J8" s="16"/>
       <c r="K8" s="12">
@@ -1502,8 +1564,9 @@
       <c r="Q8" s="13"/>
       <c r="R8" s="13"/>
       <c r="S8" s="13"/>
-    </row>
-    <row r="9" spans="1:19" ht="29" x14ac:dyDescent="0.35">
+      <c r="T8" s="7"/>
+    </row>
+    <row r="9" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
         <v>6</v>
       </c>
@@ -1517,22 +1580,22 @@
         <v>61</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G9" s="3">
         <v>0</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="K9" s="12">
         <v>1</v>
@@ -1544,10 +1607,10 @@
         <v>1</v>
       </c>
       <c r="N9" s="13" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="O9" s="13" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="P9" s="12">
         <v>1</v>
@@ -1559,10 +1622,11 @@
         <v>1</v>
       </c>
       <c r="S9" s="1" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+        <v>155</v>
+      </c>
+      <c r="T9" s="7"/>
+    </row>
+    <row r="10" spans="1:20" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="7" t="s">
         <v>7</v>
       </c>
@@ -1576,19 +1640,19 @@
         <v>61</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G10" s="3">
         <v>1</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="J10" s="13"/>
       <c r="K10" s="12">
@@ -1602,8 +1666,11 @@
       <c r="Q10" s="13"/>
       <c r="R10" s="13"/>
       <c r="S10" s="13"/>
-    </row>
-    <row r="11" spans="1:19" ht="29" x14ac:dyDescent="0.35">
+      <c r="T10" s="7" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
         <v>8</v>
       </c>
@@ -1617,19 +1684,19 @@
         <v>61</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G11" s="3">
         <v>1</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="J11" s="13"/>
       <c r="K11" s="12">
@@ -1643,8 +1710,9 @@
       <c r="Q11" s="13"/>
       <c r="R11" s="13"/>
       <c r="S11" s="13"/>
-    </row>
-    <row r="12" spans="1:19" ht="29" x14ac:dyDescent="0.35">
+      <c r="T11" s="7"/>
+    </row>
+    <row r="12" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
         <v>34</v>
       </c>
@@ -1654,17 +1722,17 @@
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
       <c r="E12" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G12" s="3"/>
       <c r="H12" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J12" s="16"/>
       <c r="K12" s="12">
@@ -1678,8 +1746,9 @@
       <c r="Q12" s="13"/>
       <c r="R12" s="13"/>
       <c r="S12" s="13"/>
-    </row>
-    <row r="13" spans="1:19" ht="58" x14ac:dyDescent="0.35">
+      <c r="T12" s="7"/>
+    </row>
+    <row r="13" spans="1:20" ht="58" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
         <v>9</v>
       </c>
@@ -1693,22 +1762,22 @@
         <v>63</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G13" s="3">
         <v>0</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I13" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="J13" s="16" t="s">
         <v>122</v>
-      </c>
-      <c r="J13" s="16" t="s">
-        <v>125</v>
       </c>
       <c r="K13" s="12">
         <v>2</v>
@@ -1717,13 +1786,13 @@
         <v>1.2</v>
       </c>
       <c r="M13" s="13" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="N13" s="13" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="O13" s="16" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="P13" s="12">
         <v>1</v>
@@ -1735,10 +1804,11 @@
         <v>0.6</v>
       </c>
       <c r="S13" s="13" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19" ht="25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>156</v>
+      </c>
+      <c r="T13" s="7"/>
+    </row>
+    <row r="14" spans="1:20" ht="25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>24</v>
       </c>
@@ -1762,8 +1832,9 @@
       <c r="Q14" s="15"/>
       <c r="R14" s="15"/>
       <c r="S14" s="15"/>
-    </row>
-    <row r="15" spans="1:19" ht="130.5" x14ac:dyDescent="0.35">
+      <c r="T14" s="6"/>
+    </row>
+    <row r="15" spans="1:20" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
         <v>10</v>
       </c>
@@ -1777,42 +1848,43 @@
         <v>61</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G15" s="3">
         <v>1</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="J15" s="16" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="K15" s="12">
         <v>1</v>
       </c>
       <c r="L15" s="13">
-        <v>0.5</v>
+        <v>3.5</v>
       </c>
       <c r="M15" s="13">
-        <v>0.5</v>
+        <v>3.5</v>
       </c>
       <c r="N15" s="13" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="O15" s="22"/>
       <c r="P15" s="29"/>
       <c r="Q15" s="23"/>
       <c r="R15" s="23"/>
       <c r="S15" s="23"/>
-    </row>
-    <row r="16" spans="1:19" ht="29" x14ac:dyDescent="0.35">
+      <c r="T15" s="7"/>
+    </row>
+    <row r="16" spans="1:20" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
         <v>11</v>
       </c>
@@ -1826,22 +1898,22 @@
         <v>63</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G16" s="3">
         <v>1</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="J16" s="13" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="K16" s="12">
         <v>1</v>
@@ -1853,13 +1925,14 @@
         <v>1</v>
       </c>
       <c r="N16" s="13" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="O16" s="23"/>
       <c r="P16" s="29"/>
       <c r="Q16" s="23"/>
       <c r="R16" s="23"/>
       <c r="S16" s="23"/>
+      <c r="T16" s="7"/>
     </row>
     <row r="17" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A17" s="7" t="s">
@@ -1873,22 +1946,22 @@
       </c>
       <c r="D17" s="7"/>
       <c r="E17" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G17" s="3">
         <v>1</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="J17" s="16" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="K17" s="12">
         <v>1</v>
@@ -1900,16 +1973,17 @@
         <v>1</v>
       </c>
       <c r="N17" s="13" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="O17" s="22"/>
       <c r="P17" s="29"/>
       <c r="Q17" s="23"/>
       <c r="R17" s="23"/>
       <c r="S17" s="23"/>
+      <c r="T17" s="7"/>
       <c r="U17" s="25"/>
       <c r="V17" s="4" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="18" spans="1:22" ht="101.5" x14ac:dyDescent="0.35">
@@ -1926,20 +2000,20 @@
         <v>60</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G18" s="3"/>
       <c r="H18" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="J18" s="13" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="K18" s="12">
         <v>1</v>
@@ -1956,6 +2030,9 @@
       <c r="Q18" s="23"/>
       <c r="R18" s="23"/>
       <c r="S18" s="23"/>
+      <c r="T18" s="7" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A19" s="7" t="s">
@@ -1971,17 +2048,17 @@
         <v>60</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G19" s="8">
         <v>1</v>
       </c>
       <c r="H19" s="8"/>
       <c r="I19" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J19" s="16"/>
       <c r="K19" s="12"/>
@@ -1993,6 +2070,7 @@
       <c r="Q19" s="24"/>
       <c r="R19" s="24"/>
       <c r="S19" s="24"/>
+      <c r="T19" s="7"/>
     </row>
     <row r="20" spans="1:22" ht="58" x14ac:dyDescent="0.35">
       <c r="A20" s="7" t="s">
@@ -2008,19 +2086,19 @@
         <v>61</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G20" s="3">
         <v>1</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="J20" s="13"/>
       <c r="K20" s="12">
@@ -2034,6 +2112,7 @@
       <c r="Q20" s="23"/>
       <c r="R20" s="23"/>
       <c r="S20" s="23"/>
+      <c r="T20" s="7"/>
     </row>
     <row r="21" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A21" s="7" t="s">
@@ -2049,22 +2128,22 @@
         <v>61</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G21" s="3">
         <v>0</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J21" s="13" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="K21" s="12">
         <v>1</v>
@@ -2081,6 +2160,9 @@
       <c r="Q21" s="23"/>
       <c r="R21" s="23"/>
       <c r="S21" s="23"/>
+      <c r="T21" s="7" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="22" spans="1:22" ht="29" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
@@ -2106,6 +2188,7 @@
       <c r="Q22" s="15"/>
       <c r="R22" s="15"/>
       <c r="S22" s="15"/>
+      <c r="T22" s="6"/>
     </row>
     <row r="23" spans="1:22" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="7" t="s">
@@ -2121,19 +2204,19 @@
         <v>63</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G23" s="3">
         <v>0</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="J23" s="16"/>
       <c r="K23" s="12">
@@ -2147,6 +2230,9 @@
       <c r="Q23" s="13"/>
       <c r="R23" s="13"/>
       <c r="S23" s="13"/>
+      <c r="T23" s="7" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A24" s="7" t="s">
@@ -2158,10 +2244,10 @@
       <c r="C24" s="7"/>
       <c r="D24" s="7"/>
       <c r="E24" s="8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="G24" s="8">
         <v>0</v>
@@ -2178,6 +2264,7 @@
       <c r="Q24" s="16"/>
       <c r="R24" s="16"/>
       <c r="S24" s="16"/>
+      <c r="T24" s="7"/>
     </row>
     <row r="25" spans="1:22" ht="58" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
@@ -2193,22 +2280,22 @@
         <v>60</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G25" s="3">
         <v>1</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="J25" s="16" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="K25" s="12">
         <v>1</v>
@@ -2220,13 +2307,14 @@
         <v>1</v>
       </c>
       <c r="N25" s="4" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="O25" s="16"/>
       <c r="P25" s="12"/>
       <c r="Q25" s="13"/>
       <c r="R25" s="13"/>
       <c r="S25" s="7"/>
+      <c r="T25" s="7"/>
     </row>
     <row r="26" spans="1:22" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="7" t="s">
@@ -2242,17 +2330,19 @@
         <v>60</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G26" s="8">
-        <v>1</v>
-      </c>
-      <c r="H26" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="H26" s="8" t="s">
+        <v>167</v>
+      </c>
       <c r="I26" s="8" t="s">
-        <v>69</v>
+        <v>168</v>
       </c>
       <c r="J26" s="16"/>
       <c r="K26" s="12">
@@ -2266,6 +2356,9 @@
       <c r="Q26" s="13"/>
       <c r="R26" s="13"/>
       <c r="S26" s="13"/>
+      <c r="T26" s="7" t="s">
+        <v>170</v>
+      </c>
     </row>
     <row r="27" spans="1:22" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A27" s="7" t="s">
@@ -2281,22 +2374,22 @@
         <v>60</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G27" s="3">
         <v>0</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="J27" s="13" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="K27" s="12">
         <v>2</v>
@@ -2305,13 +2398,13 @@
         <v>1.2</v>
       </c>
       <c r="M27" s="13" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="N27" s="13" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="O27" s="13" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="P27" s="12">
         <v>1</v>
@@ -2323,8 +2416,9 @@
         <v>1</v>
       </c>
       <c r="S27" s="7" t="s">
-        <v>163</v>
-      </c>
+        <v>159</v>
+      </c>
+      <c r="T27" s="7"/>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A28" s="7" t="s">
@@ -2340,17 +2434,19 @@
         <v>60</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G28" s="8">
-        <v>1</v>
-      </c>
-      <c r="H28" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="H28" s="8" t="s">
+        <v>167</v>
+      </c>
       <c r="I28" s="8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J28" s="16"/>
       <c r="K28" s="12">
@@ -2364,6 +2460,9 @@
       <c r="Q28" s="13"/>
       <c r="R28" s="13"/>
       <c r="S28" s="13"/>
+      <c r="T28" s="7" t="s">
+        <v>171</v>
+      </c>
     </row>
     <row r="29" spans="1:22" ht="58" x14ac:dyDescent="0.35">
       <c r="A29" s="7" t="s">
@@ -2379,19 +2478,19 @@
         <v>60</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G29" s="3">
         <v>1</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="J29" s="16"/>
       <c r="K29" s="12">
@@ -2405,6 +2504,7 @@
       <c r="Q29" s="13"/>
       <c r="R29" s="13"/>
       <c r="S29" s="13"/>
+      <c r="T29" s="7"/>
     </row>
     <row r="30" spans="1:22" ht="29" x14ac:dyDescent="0.35">
       <c r="A30" s="7" t="s">
@@ -2418,20 +2518,20 @@
         <v>60</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G30" s="3"/>
       <c r="H30" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="J30" s="16" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="K30" s="12">
         <v>1</v>
@@ -2443,10 +2543,10 @@
         <v>1</v>
       </c>
       <c r="N30" s="13" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="O30" s="16" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="P30" s="12">
         <v>1</v>
@@ -2458,8 +2558,9 @@
         <v>1</v>
       </c>
       <c r="S30" s="1" t="s">
-        <v>161</v>
-      </c>
+        <v>157</v>
+      </c>
+      <c r="T30" s="7"/>
     </row>
     <row r="31" spans="1:22" ht="26" x14ac:dyDescent="0.35">
       <c r="A31" s="7"/>
@@ -2471,7 +2572,7 @@
       <c r="G31" s="7"/>
       <c r="H31" s="7"/>
       <c r="I31" s="7" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="J31" s="20"/>
       <c r="K31" s="19">
@@ -2480,7 +2581,7 @@
       </c>
       <c r="L31" s="21">
         <f>SUM(L2:L30)</f>
-        <v>10.199999999999999</v>
+        <v>15.2</v>
       </c>
       <c r="M31" s="21"/>
       <c r="N31" s="21"/>
@@ -2495,6 +2596,7 @@
       </c>
       <c r="R31" s="21"/>
       <c r="S31" s="21"/>
+      <c r="T31" s="7"/>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.35">
       <c r="B33" s="10" t="s">

</xml_diff>